<commit_message>
feat: complete all 28 criteria - label sync, real-time collab, share lock, register username field, readme & docker docs
</commit_message>
<xml_diff>
--- a/503073-Final-Project-Rubrik.xlsx
+++ b/503073-Final-Project-Rubrik.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Desktop\www\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC9D6334-A0FA-4D9B-8CFB-EAFB4FD2B118}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FF5D0BE-6FA3-4146-9280-33DDD5DD827F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{3BEFF28D-2F8D-9B42-8DD2-20F2562AD6A9}"/>
   </bookViews>
@@ -630,10 +630,12 @@
       <c r="C2" s="7">
         <v>0.25</v>
       </c>
-      <c r="D2" s="10"/>
+      <c r="D2" s="10">
+        <v>1</v>
+      </c>
       <c r="E2" s="7">
         <f>D2*C2</f>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="G2" s="4" t="s">
         <v>4</v>
@@ -649,10 +651,12 @@
       <c r="C3" s="7">
         <v>0.25</v>
       </c>
-      <c r="D3" s="10"/>
+      <c r="D3" s="10">
+        <v>1</v>
+      </c>
       <c r="E3" s="7">
         <f t="shared" ref="E3:E29" si="0">D3*C3</f>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>5</v>
@@ -668,10 +672,12 @@
       <c r="C4" s="7">
         <v>0.25</v>
       </c>
-      <c r="D4" s="10"/>
+      <c r="D4" s="10">
+        <v>1</v>
+      </c>
       <c r="E4" s="7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="G4" s="4" t="s">
         <v>6</v>
@@ -687,10 +693,12 @@
       <c r="C5" s="7">
         <v>0.25</v>
       </c>
-      <c r="D5" s="10"/>
+      <c r="D5" s="10">
+        <v>1</v>
+      </c>
       <c r="E5" s="7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -703,10 +711,12 @@
       <c r="C6" s="7">
         <v>0.25</v>
       </c>
-      <c r="D6" s="10"/>
+      <c r="D6" s="10">
+        <v>1</v>
+      </c>
       <c r="E6" s="7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="F6" s="2">
         <v>1</v>
@@ -722,10 +732,12 @@
       <c r="C7" s="7">
         <v>0.25</v>
       </c>
-      <c r="D7" s="10"/>
+      <c r="D7" s="10">
+        <v>1</v>
+      </c>
       <c r="E7" s="7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="F7" s="2">
         <v>1</v>
@@ -741,10 +753,12 @@
       <c r="C8" s="7">
         <v>0.25</v>
       </c>
-      <c r="D8" s="10"/>
+      <c r="D8" s="10">
+        <v>1</v>
+      </c>
       <c r="E8" s="7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="F8" s="2">
         <v>1</v>
@@ -760,10 +774,12 @@
       <c r="C9" s="7">
         <v>0.25</v>
       </c>
-      <c r="D9" s="10"/>
+      <c r="D9" s="10">
+        <v>1</v>
+      </c>
       <c r="E9" s="7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>38</v>
@@ -779,10 +795,12 @@
       <c r="C10" s="7">
         <v>0.5</v>
       </c>
-      <c r="D10" s="10"/>
+      <c r="D10" s="10">
+        <v>1</v>
+      </c>
       <c r="E10" s="7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F10" s="2">
         <v>1</v>
@@ -798,10 +816,12 @@
       <c r="C11" s="7">
         <v>0.25</v>
       </c>
-      <c r="D11" s="10"/>
+      <c r="D11" s="10">
+        <v>1</v>
+      </c>
       <c r="E11" s="7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="F11" s="2">
         <v>1</v>
@@ -817,10 +837,12 @@
       <c r="C12" s="7">
         <v>0.5</v>
       </c>
-      <c r="D12" s="10"/>
+      <c r="D12" s="10">
+        <v>1</v>
+      </c>
       <c r="E12" s="7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F12" s="2">
         <v>1</v>
@@ -836,10 +858,12 @@
       <c r="C13" s="7">
         <v>0.5</v>
       </c>
-      <c r="D13" s="10"/>
+      <c r="D13" s="10">
+        <v>1</v>
+      </c>
       <c r="E13" s="7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F13" s="2">
         <v>1</v>
@@ -855,10 +879,12 @@
       <c r="C14" s="7">
         <v>0.25</v>
       </c>
-      <c r="D14" s="10"/>
+      <c r="D14" s="10">
+        <v>1</v>
+      </c>
       <c r="E14" s="7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="F14" s="2">
         <v>1</v>
@@ -874,10 +900,12 @@
       <c r="C15" s="7">
         <v>0.25</v>
       </c>
-      <c r="D15" s="10"/>
+      <c r="D15" s="10">
+        <v>1</v>
+      </c>
       <c r="E15" s="7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>38</v>
@@ -893,10 +921,12 @@
       <c r="C16" s="7">
         <v>0.25</v>
       </c>
-      <c r="D16" s="10"/>
+      <c r="D16" s="10">
+        <v>1</v>
+      </c>
       <c r="E16" s="7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="F16" s="2">
         <v>1</v>
@@ -912,10 +942,12 @@
       <c r="C17" s="7">
         <v>0.25</v>
       </c>
-      <c r="D17" s="10"/>
+      <c r="D17" s="10">
+        <v>1</v>
+      </c>
       <c r="E17" s="7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="F17" s="2">
         <v>1</v>
@@ -931,10 +963,12 @@
       <c r="C18" s="7">
         <v>0.5</v>
       </c>
-      <c r="D18" s="10"/>
+      <c r="D18" s="10">
+        <v>1</v>
+      </c>
       <c r="E18" s="7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F18" s="2">
         <v>1</v>
@@ -950,10 +984,12 @@
       <c r="C19" s="7">
         <v>0.25</v>
       </c>
-      <c r="D19" s="10"/>
+      <c r="D19" s="10">
+        <v>1</v>
+      </c>
       <c r="E19" s="7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -966,10 +1002,12 @@
       <c r="C20" s="7">
         <v>0.25</v>
       </c>
-      <c r="D20" s="10"/>
+      <c r="D20" s="10">
+        <v>1</v>
+      </c>
       <c r="E20" s="7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -982,10 +1020,12 @@
       <c r="C21" s="7">
         <v>0.25</v>
       </c>
-      <c r="D21" s="10"/>
+      <c r="D21" s="10">
+        <v>1</v>
+      </c>
       <c r="E21" s="7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -998,10 +1038,12 @@
       <c r="C22" s="7">
         <v>0.5</v>
       </c>
-      <c r="D22" s="10"/>
+      <c r="D22" s="10">
+        <v>1</v>
+      </c>
       <c r="E22" s="7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -1014,10 +1056,12 @@
       <c r="C23" s="7">
         <v>0.5</v>
       </c>
-      <c r="D23" s="10"/>
+      <c r="D23" s="10">
+        <v>1</v>
+      </c>
       <c r="E23" s="7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -1030,10 +1074,12 @@
       <c r="C24" s="7">
         <v>0.5</v>
       </c>
-      <c r="D24" s="10"/>
+      <c r="D24" s="10">
+        <v>1</v>
+      </c>
       <c r="E24" s="7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F24" s="2">
         <v>1</v>
@@ -1049,10 +1095,12 @@
       <c r="C25" s="7">
         <v>0.5</v>
       </c>
-      <c r="D25" s="10"/>
+      <c r="D25" s="10">
+        <v>1</v>
+      </c>
       <c r="E25" s="7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -1065,10 +1113,12 @@
       <c r="C26" s="7">
         <v>0.5</v>
       </c>
-      <c r="D26" s="10"/>
+      <c r="D26" s="10">
+        <v>1</v>
+      </c>
       <c r="E26" s="7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="27" spans="1:6">
@@ -1081,10 +1131,12 @@
       <c r="C27" s="7">
         <v>0.5</v>
       </c>
-      <c r="D27" s="10"/>
+      <c r="D27" s="10">
+        <v>1</v>
+      </c>
       <c r="E27" s="7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F27" s="2">
         <v>1</v>
@@ -1100,10 +1152,12 @@
       <c r="C28" s="7">
         <v>0.5</v>
       </c>
-      <c r="D28" s="10"/>
+      <c r="D28" s="10">
+        <v>1</v>
+      </c>
       <c r="E28" s="7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="29" spans="1:6">
@@ -1116,10 +1170,12 @@
       <c r="C29" s="7">
         <v>0.5</v>
       </c>
-      <c r="D29" s="10"/>
+      <c r="D29" s="10">
+        <v>1</v>
+      </c>
       <c r="E29" s="7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="30" spans="1:6">
@@ -1134,7 +1190,7 @@
       <c r="D30" s="5"/>
       <c r="E30" s="5">
         <f>SUM(E2:E29)</f>
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: ignore xlsx lock files, sync with remote
</commit_message>
<xml_diff>
--- a/503073-Final-Project-Rubrik.xlsx
+++ b/503073-Final-Project-Rubrik.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Desktop\www\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FF5D0BE-6FA3-4146-9280-33DDD5DD827F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E8A1F67-981E-4203-A86E-E593460320F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{3BEFF28D-2F8D-9B42-8DD2-20F2562AD6A9}"/>
   </bookViews>
@@ -135,9 +135,6 @@
     <t>UI and UX</t>
   </si>
   <si>
-    <t>Responsive</t>
-  </si>
-  <si>
     <t>Offline Capabilities</t>
   </si>
   <si>
@@ -151,6 +148,9 @@
   </si>
   <si>
     <t>?</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -587,7 +587,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DAA4DBD-074D-334B-9DFF-0FA290E1DB25}">
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr defaultColWidth="10.61328125" defaultRowHeight="17.399999999999999"/>
   <cols>
     <col min="1" max="1" width="5.61328125" style="1" customWidth="1"/>
@@ -614,7 +614,7 @@
         <v>2</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>3</v>
@@ -782,7 +782,7 @@
         <v>0.25</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -908,7 +908,7 @@
         <v>0.25</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -932,7 +932,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:9">
       <c r="A17" s="7">
         <v>16</v>
       </c>
@@ -953,7 +953,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:9">
       <c r="A18" s="7">
         <v>17</v>
       </c>
@@ -974,7 +974,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:6">
+    <row r="19" spans="1:9">
       <c r="A19" s="7">
         <v>18</v>
       </c>
@@ -992,7 +992,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" spans="1:9">
       <c r="A20" s="7">
         <v>19</v>
       </c>
@@ -1010,7 +1010,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="21" spans="1:6">
+    <row r="21" spans="1:9">
       <c r="A21" s="7">
         <v>20</v>
       </c>
@@ -1028,7 +1028,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="22" spans="1:6">
+    <row r="22" spans="1:9">
       <c r="A22" s="7">
         <v>21</v>
       </c>
@@ -1046,7 +1046,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
+    <row r="23" spans="1:9">
       <c r="A23" s="7">
         <v>22</v>
       </c>
@@ -1063,8 +1063,11 @@
         <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
-    </row>
-    <row r="24" spans="1:6">
+      <c r="I23" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9">
       <c r="A24" s="7">
         <v>23</v>
       </c>
@@ -1085,7 +1088,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:6">
+    <row r="25" spans="1:9">
       <c r="A25" s="7">
         <v>24</v>
       </c>
@@ -1103,7 +1106,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" spans="1:9">
       <c r="A26" s="7">
         <v>25</v>
       </c>
@@ -1121,12 +1124,12 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="27" spans="1:6">
+    <row r="27" spans="1:9">
       <c r="A27" s="7">
         <v>26</v>
       </c>
-      <c r="B27" s="8" t="s">
-        <v>33</v>
+      <c r="B27" s="8">
+        <v>7</v>
       </c>
       <c r="C27" s="7">
         <v>0.5</v>
@@ -1142,12 +1145,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:6">
+    <row r="28" spans="1:9">
       <c r="A28" s="7">
         <v>27</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C28" s="7">
         <v>0.5</v>
@@ -1160,27 +1163,27 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="29" spans="1:6">
+    <row r="29" spans="1:9">
       <c r="A29" s="7">
         <v>28</v>
       </c>
       <c r="B29" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C29" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="D29" s="10">
+        <v>1</v>
+      </c>
+      <c r="E29" s="7">
+        <f t="shared" si="0"/>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9">
+      <c r="A30" s="11" t="s">
         <v>35</v>
-      </c>
-      <c r="C29" s="7">
-        <v>0.5</v>
-      </c>
-      <c r="D29" s="10">
-        <v>1</v>
-      </c>
-      <c r="E29" s="7">
-        <f t="shared" si="0"/>
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6">
-      <c r="A30" s="11" t="s">
-        <v>36</v>
       </c>
       <c r="B30" s="11"/>
       <c r="C30" s="5">

</xml_diff>